<commit_message>
Chart: whole-number axis labels and drop redundant x-axis title
- Set both axes to numFmt '0' with sourceLinked=false so tick labels render
  as 0/20/40/60/80/100 instead of inheriting the cells' '0.0' format, which
  displayed as '100,0' under comma-decimal locales
- Remove the 'Index year' axis title, which collided with the 2021/2022
  tick labels at this figure size

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018p7yWaMxvZssm82Ne1xPhx
</commit_message>
<xml_diff>
--- a/Property_Rights_2017_2026.xlsx
+++ b/Property_Rights_2017_2026.xlsx
@@ -400,21 +400,7 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Index year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -446,6 +432,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>

</xml_diff>

<commit_message>
Chart: give the y-axis title clearance from its tick labels
Auto-layout crowded the rotated axis title against the 0-100 tick labels at
11 cm wide. Place the plot area explicitly with a 17% left margin, pin the
title to the left edge, and set axis text to 9 pt Arial (legend 8.5 pt) so
the furniture needs less room.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018p7yWaMxvZssm82Ne1xPhx
</commit_message>
<xml_diff>
--- a/Property_Rights_2017_2026.xlsx
+++ b/Property_Rights_2017_2026.xlsx
@@ -208,6 +208,18 @@
       </tx>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.17"/>
+          <y val="0.11"/>
+          <w val="0.79"/>
+          <h val="0.62"/>
+        </manualLayout>
+      </layout>
       <lineChart>
         <grouping val="standard"/>
         <ser>
@@ -403,6 +415,22 @@
         <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="900" b="0">
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
@@ -423,7 +451,9 @@
               <a:bodyPr/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr/>
+                  <a:defRPr sz="900">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
                 </a:pPr>
                 <a:r>
                   <a:t>Property rights score (0–100)</a:t>
@@ -431,10 +461,36 @@
               </a:p>
             </rich>
           </tx>
+          <layout>
+            <manualLayout>
+              <xMode val="edge"/>
+              <yMode val="edge"/>
+              <wMode val="factor"/>
+              <hMode val="factor"/>
+              <x val="0.005"/>
+              <y val="0.16"/>
+            </manualLayout>
+          </layout>
         </title>
         <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="900" b="0">
+              <a:latin typeface="Arial"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
         <majorUnit val="20"/>
       </valAx>
@@ -442,6 +498,22 @@
     <legend>
       <legendPos val="b"/>
       <overlay val="0"/>
+      <txPr>
+        <a:bodyPr/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="850" b="0">
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr sz="850" b="0">
+            <a:latin typeface="Arial"/>
+          </a:endParaRPr>
+        </a:p>
+      </txPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>

</xml_diff>